<commit_message>
Select three 2TB PC801 SSDs for Berserk RAID 0
</commit_message>
<xml_diff>
--- a/parts.xlsx
+++ b/parts.xlsx
@@ -812,7 +812,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -1219,31 +1219,31 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
-        <is>
-          <t>Samsung 960 PRO 1 TB NVMe</t>
-        </is>
+    <row r="13" ht="48" customHeight="1">
+      <c r="A13" s="1" t="str">
+        <v>SK hynix PC801 2 TB NVMe (HFS002TEJ9X101NFC)</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
           <t>each</t>
         </is>
       </c>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2">
+      <c r="D13" s="2" t="n">
+        <v>204.99</v>
+      </c>
+      <c r="E13" s="2" t="n">
         <f>IF(OR(B13="",D13=""),"",B13*D13)</f>
-        <v/>
-      </c>
-      <c r="F13" s="1" t="n"/>
+        <v>614.97</v>
+      </c>
+      <c r="F13" s="1" t="str">
+        <v>eBay listing</v>
+      </c>
       <c r="G13" s="1" t="inlineStr"/>
-      <c r="H13" s="1" t="inlineStr">
-        <is>
-          <t>Reused.</t>
-        </is>
+      <c r="H13" s="1" t="str">
+        <v>3-drive RAID 0, 6 TB nominal. Used; seller reports 100% health. Free US shipping, tax extra (2026-10-22). All M.2 slots occupied; boot layout and SSD cooling/clearance unverified.</v>
       </c>
     </row>
     <row r="14">
@@ -1306,25 +1306,26 @@
           <t>Known total</t>
         </is>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="5" t="n">
         <f>SUM(E2:E15)</f>
-        <v/>
+        <v>2134.63</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId8"/>
+    <hyperlink ref="F2" r:id="rId1"/>
+    <hyperlink ref="F4" r:id="rId2"/>
+    <hyperlink ref="F5" r:id="rId3"/>
+    <hyperlink ref="F6" r:id="rId4"/>
+    <hyperlink ref="F7" r:id="rId5"/>
+    <hyperlink ref="F8" r:id="rId6"/>
+    <hyperlink ref="F9" r:id="rId7"/>
+    <hyperlink ref="F10" r:id="rId8"/>
+    <hyperlink ref="F13" r:id="rIdSSDListing"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId9"/>
+    <tablePart r:id="rId9"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Mount GPU posts through snug hex holes directly to steel
Use 14 mm M3 through-thread bases and M3x6 underside screws to clear the owner-reported 9 mm OBT studs. Locate the bases with regular 5.8 mm hex openings and retain each adapter with five independent shelf anchors.

Regenerate CAD, print plates, previews and fit reports; update assembly guidance and the parts workbook. CAD checks, all 14 support-free slices and the independent prototype print audit passed. Actual hardware fit remains provisional.
</commit_message>
<xml_diff>
--- a/parts.xlsx
+++ b/parts.xlsx
@@ -486,329 +486,324 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="90" customWidth="1" min="8" max="8"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Unit price (USD)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Total (USD)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>More links</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
-        <is>
-          <t>StarTech ADJSHELFHDV 1U four-post vented shelf</t>
-        </is>
-      </c>
-      <c r="B2" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="n">
-        <v>166.13</v>
-      </c>
-      <c r="E2" s="2">
-        <f>IF(OR(B2="",D2=""),"",B2*D2)</f>
-        <v/>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G2" s="1" t="inlineStr"/>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>700 × 446 mm steel deck. The build drills new mounting holes into it; survey the real lips, vents and cabinet liners first.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
-        <is>
-          <t>Keystone 1451B #6-32 F/F brass standoff, 3/8 in (9.53 mm)</t>
-        </is>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>17</v>
-      </c>
-      <c r="C3" s="1" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n">
-        <v>0.88</v>
-      </c>
-      <c r="E3" s="2">
-        <f>IF(OR(B3="",D3=""),"",B3*D3)</f>
-        <v/>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>Eight for the H12D, nine for the X870E. Fit only the board's populated holes; ground one standoff to the shelf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
-        <is>
-          <t>Open Benchtable PCI-E support + nut, 2-pack</t>
-        </is>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" s="1" t="inlineStr">
-        <is>
-          <t>2-pack</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E4" s="2">
-        <f>IF(OR(B4="",D4=""),"",B4*D4)</f>
-        <v/>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Open Benchtable</t>
-        </is>
-      </c>
-      <c r="G4" s="1" t="inlineStr"/>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>Ten metal posts, two per GPU, for five GPUs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Würth 970100354 M3 F/F brass standoff, 10 mm</t>
-        </is>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C5" s="1" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="E5" s="2">
-        <f>IF(OR(B5="",D5=""),"",B5*D5)</f>
-        <v/>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G5" s="1" t="inlineStr"/>
-      <c r="H5" s="1" t="inlineStr">
-        <is>
-          <t>One under each GPU post; clamps the post and the motherboard adapter to the steel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
-        <is>
-          <t>Shelf fasteners and backing washers</t>
-        </is>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>39</v>
-      </c>
-      <c r="C6" s="1" t="inlineStr">
-        <is>
-          <t>joints</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2">
-        <f>IF(OR(B6="",D6=""),"",B6*D6)</f>
-        <v/>
-      </c>
-      <c r="F6" s="1" t="n"/>
-      <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr">
-        <is>
-          <t>25 M4 joints (21 printed mounts, four V100 tail spacers) and 14 M3 joints (four front motherboard anchors, ten GPU-post joints). Stacks and lengths are in mount-hole-manifest.json and the assembly guide.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>Component fasteners and interface hardware</t>
-        </is>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="inlineStr">
-        <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2">
-        <f>IF(OR(B7="",D7=""),"",B7*D7)</f>
-        <v/>
-      </c>
-      <c r="F7" s="1" t="n"/>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr">
-        <is>
-          <t>17 low-head #6-32 standoff screws, PSU and radiator screws, four M4 × 20 mm F/F metal tail spacers with 4 mm silicone pads, nonconductive foam seal for the GPU hood.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>AC power cords</t>
-        </is>
-      </c>
-      <c r="B8" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" s="1" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2">
-        <f>IF(OR(B8="",D8=""),"",B8*D8)</f>
-        <v/>
-      </c>
-      <c r="F8" s="1" t="n"/>
-      <c r="G8" s="1" t="inlineStr"/>
-      <c r="H8" s="1" t="inlineStr">
-        <is>
-          <t>Corsair: low-profile or down-exit C13. Rosewill: match its inlet and the UPS outlet (it may need C19).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>Printed parts</t>
-        </is>
-      </c>
-      <c r="B9" s="1" t="n">
-        <v>18</v>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>each</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2">
-        <f>IF(OR(B9="",D9=""),"",B9*D9)</f>
-        <v/>
-      </c>
-      <c r="F9" s="1" t="n"/>
-      <c r="G9" s="1" t="inlineStr"/>
-      <c r="H9" s="1" t="inlineStr">
-        <is>
-          <t>17 installed parts plus one fit coupon, on 14 plates. See print/README.md.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Known total</t>
-        </is>
-      </c>
-      <c r="E11" s="5">
-        <f>SUM(E2:E9)</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId4"/>
-  </hyperlinks>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
-  </tableParts>
-</worksheet>
+<ns0:worksheet xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:sheetPr>
+    <ns0:outlinePr summaryBelow="1" summaryRight="1"/>
+    <ns0:pageSetUpPr/>
+  </ns0:sheetPr>
+  <ns0:dimension ref="A1:H11"/>
+  <ns0:sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <ns0:cols>
+    <ns0:col width="48" customWidth="1" min="1" max="1"/>
+    <ns0:col width="7" customWidth="1" min="2" max="2"/>
+    <ns0:col width="9" customWidth="1" min="3" max="3"/>
+    <ns0:col width="14" customWidth="1" min="4" max="4"/>
+    <ns0:col width="12" customWidth="1" min="5" max="5"/>
+    <ns0:col width="16" customWidth="1" min="6" max="6"/>
+    <ns0:col width="40" customWidth="1" min="7" max="7"/>
+    <ns0:col width="90" customWidth="1" min="8" max="8"/>
+  </ns0:cols>
+  <ns0:sheetData>
+    <ns0:row r="1">
+      <ns0:c r="A1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Item</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Qty</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="C1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Unit</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Unit price (USD)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Total (USD)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="F1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Link</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>More links</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="H1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Notes</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="2">
+      <ns0:c r="A2" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>StarTech ADJSHELFHDV 1U four-post vented shelf</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B2" s="1" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="C2" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>each</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D2" s="2" t="n">
+        <ns0:v>166.13</ns0:v>
+      </ns0:c>
+      <ns0:c r="E2" s="2">
+        <ns0:f>IF(OR(B2="",D2=""),"",B2*D2)</ns0:f>
+        <ns0:v/>
+      </ns0:c>
+      <ns0:c r="F2" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DigiKey</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G2" s="1" t="inlineStr"/>
+      <ns0:c r="H2" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>700 × 446 mm steel deck. The build drills new mounting holes into it; survey the real lips, vents and cabinet liners first.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="3">
+      <ns0:c r="A3" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Keystone 1451B #6-32 F/F brass standoff, 3/8 in (9.53 mm)</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B3" s="1" t="n">
+        <ns0:v>17</ns0:v>
+      </ns0:c>
+      <ns0:c r="C3" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>each</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D3" s="2" t="n">
+        <ns0:v>0.88</ns0:v>
+      </ns0:c>
+      <ns0:c r="E3" s="2">
+        <ns0:f>IF(OR(B3="",D3=""),"",B3*D3)</ns0:f>
+        <ns0:v/>
+      </ns0:c>
+      <ns0:c r="F3" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DigiKey</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G3" s="1" t="inlineStr"/>
+      <ns0:c r="H3" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Eight for the H12D, nine for the X870E. Fit only the board's populated holes; ground one standoff to the shelf.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="4" ht="28" customHeight="1">
+      <ns0:c r="A4" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Open Benchtable PCI-E support + nut, 2-pack</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B4" s="1" t="n">
+        <ns0:v>5</ns0:v>
+      </ns0:c>
+      <ns0:c r="C4" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>2-pack</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D4" s="2" t="n">
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="E4" s="2">
+        <ns0:f>IF(OR(B4="",D4=""),"",B4*D4)</ns0:f>
+        <ns0:v/>
+      </ns0:c>
+      <ns0:c r="F4" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Open Benchtable</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G4" s="1" t="inlineStr"/>
+      <ns0:c r="H4" s="1" t="str">
+        <ns0:v>Ten posts, two per GPU. Owner reports 9 mm male M3 tips; fixed lower-nut height needs dry-fit.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="5" ht="44" customHeight="1">
+      <ns0:c r="A5" s="1" t="str">
+        <ns0:v>Würth 970140324 M3 F/F brass standoff, 14 mm</ns0:v>
+      </ns0:c>
+      <ns0:c r="B5" s="1" t="n">
+        <ns0:v>10</ns0:v>
+      </ns0:c>
+      <ns0:c r="C5" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>each</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D5" s="2" t="n">
+        <ns0:v>0.635</ns0:v>
+      </ns0:c>
+      <ns0:c r="E5" s="2" t="n">
+        <ns0:f>IF(OR(B5="",D5=""),"",B5*D5)</ns0:f>
+        <ns0:v>6.35</ns0:v>
+      </ns0:c>
+      <ns0:c r="F5" s="3" t="inlineStr">
+        <ns0:is>
+          <ns0:t>DigiKey</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="G5" s="1" t="str">
+        <ns0:v>Manufacturer drawing</ns0:v>
+      </ns0:c>
+      <ns0:c r="H5" s="1" t="str">
+        <ns0:v>Ten replacement bases, SW5.5, full M3 thread. Pass through plastic to steel. M3x6 below gives 3.3 mm nominal engagement and 1.7 mm gap to 9 mm OBT stud. DigiKey price at qty10, checked 2026-10-23. Height needs dry-fit.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="6" ht="44" customHeight="1">
+      <ns0:c r="A6" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Shelf fasteners and backing washers</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B6" s="1" t="n">
+        <ns0:v>45</ns0:v>
+      </ns0:c>
+      <ns0:c r="C6" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>joints</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D6" s="2" t="n"/>
+      <ns0:c r="E6" s="2">
+        <ns0:f>IF(OR(B6="",D6=""),"",B6*D6)</ns0:f>
+        <ns0:v/>
+      </ns0:c>
+      <ns0:c r="F6" s="1" t="n"/>
+      <ns0:c r="G6" s="1" t="inlineStr"/>
+      <ns0:c r="H6" s="1" t="str">
+        <ns0:v>25 M4 joints and 20 M3 joints: ten adapter anchors (M3x16, OD7 top/back washers, nuts), ten GPU bases (M3x6, OD7 + OD12 underside washers). Six adapter anchors go in before the PCB. See assembly guide.</ns0:v>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="7">
+      <ns0:c r="A7" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Component fasteners and interface hardware</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B7" s="1" t="n">
+        <ns0:v>1</ns0:v>
+      </ns0:c>
+      <ns0:c r="C7" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>set</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D7" s="2" t="n"/>
+      <ns0:c r="E7" s="2">
+        <ns0:f>IF(OR(B7="",D7=""),"",B7*D7)</ns0:f>
+        <ns0:v/>
+      </ns0:c>
+      <ns0:c r="F7" s="1" t="n"/>
+      <ns0:c r="G7" s="1" t="inlineStr"/>
+      <ns0:c r="H7" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>17 low-head #6-32 standoff screws, PSU and radiator screws, four M4 × 20 mm F/F metal tail spacers with 4 mm silicone pads, nonconductive foam seal for the GPU hood.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="8">
+      <ns0:c r="A8" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>AC power cords</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B8" s="1" t="n">
+        <ns0:v>2</ns0:v>
+      </ns0:c>
+      <ns0:c r="C8" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>each</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D8" s="2" t="n"/>
+      <ns0:c r="E8" s="2">
+        <ns0:f>IF(OR(B8="",D8=""),"",B8*D8)</ns0:f>
+        <ns0:v/>
+      </ns0:c>
+      <ns0:c r="F8" s="1" t="n"/>
+      <ns0:c r="G8" s="1" t="inlineStr"/>
+      <ns0:c r="H8" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Corsair: low-profile or down-exit C13. Rosewill: match its inlet and the UPS outlet (it may need C19).</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="9">
+      <ns0:c r="A9" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Printed parts</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="B9" s="1" t="n">
+        <ns0:v>18</ns0:v>
+      </ns0:c>
+      <ns0:c r="C9" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>each</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="D9" s="2" t="n"/>
+      <ns0:c r="E9" s="2">
+        <ns0:f>IF(OR(B9="",D9=""),"",B9*D9)</ns0:f>
+        <ns0:v/>
+      </ns0:c>
+      <ns0:c r="F9" s="1" t="n"/>
+      <ns0:c r="G9" s="1" t="inlineStr"/>
+      <ns0:c r="H9" s="1" t="inlineStr">
+        <ns0:is>
+          <ns0:t>17 installed parts plus one fit coupon, on 14 plates. See print/README.md.</ns0:t>
+        </ns0:is>
+      </ns0:c>
+    </ns0:row>
+    <ns0:row r="11">
+      <ns0:c r="A11" s="4" t="inlineStr">
+        <ns0:is>
+          <ns0:t>Known total</ns0:t>
+        </ns0:is>
+      </ns0:c>
+      <ns0:c r="E11" s="5" t="n">
+        <ns0:f>SUM(E2:E9)</ns0:f>
+        <ns0:v>237.44</ns0:v>
+      </ns0:c>
+    </ns0:row>
+  </ns0:sheetData>
+  <ns0:hyperlinks>
+    <ns0:hyperlink ref="F2" ns1:id="rId1"/>
+    <ns0:hyperlink ref="F3" ns1:id="rId2"/>
+    <ns0:hyperlink ref="F4" ns1:id="rId3"/>
+    <ns0:hyperlink ref="F5" ns1:id="rId4"/>
+    <ns0:hyperlink ref="G5" ns1:id="rIdGpuBaseDrawing"/>
+  </ns0:hyperlinks>
+  <ns0:pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <ns0:tableParts count="1">
+    <ns0:tablePart ns1:id="rId5"/>
+  </ns0:tableParts>
+</ns0:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>